<commit_message>
Correct bottle row to Tatuo 12-pack (qty 1 pack)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WZy7dLHhGnzbT4xp7nPVJM
</commit_message>
<xml_diff>
--- a/TA_Order_List.xlsx
+++ b/TA_Order_List.xlsx
@@ -591,7 +591,7 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>1000 mL wide-mouth PP bottles, leak-proof screw cap</t>
+          <t>1000 mL polypropylene bottles with screw caps, 12-pack (Tatuo)</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
@@ -601,16 +601,16 @@
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>B07DHWGFJM</t>
+          <t>see link</t>
         </is>
       </c>
       <c r="E5" s="4" t="inlineStr">
         <is>
-          <t>1 bottle</t>
+          <t>12 bottles</t>
         </is>
       </c>
       <c r="F5" s="5" t="n">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="G5" s="6" t="n"/>
       <c r="H5" s="7">
@@ -624,7 +624,7 @@
       </c>
       <c r="J5" s="4" t="inlineStr">
         <is>
-          <t>Oxygenation test vessel. Earlier listing: $5.99 each.</t>
+          <t>1 pack = 12 bottles. Each bottle 3.54 in (~90 mm) W × 7.8 in (~198 mm) H, polypropylene. Enter the pack price.</t>
         </is>
       </c>
     </row>

</xml_diff>